<commit_message>
Python - Aula 294. Criando Emails em Massa com Python e Gmail
</commit_message>
<xml_diff>
--- a/TKinter/EmailAniversarios/Aniversario.xlsx
+++ b/TKinter/EmailAniversarios/Aniversario.xlsx
@@ -166,15 +166,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -467,7 +467,7 @@
         <v>5</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>34837</v>
+        <v>34838</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>6</v>
@@ -500,7 +500,7 @@
         <v>11</v>
       </c>
       <c r="B6" s="3" t="n">
-        <v>37029</v>
+        <v>37030</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>12</v>

</xml_diff>